<commit_message>
updated graphs to new biocro with biocrowater, changed the simulation to start from seed (DVI=-1)
</commit_message>
<xml_diff>
--- a/Data/2022_Carb_data/LD11_All.xlsx
+++ b/Data/2022_Carb_data/LD11_All.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ximinpiao/Documents/GitHub/UTR-Soybean-BioCro/Data/2022_Carb_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAE9555D-BA93-0C40-A95B-82FF4EEB68B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CD917B3-2656-8040-B758-28923A9F79F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16380" xr2:uid="{AD88AA4B-C132-0C4D-B7C9-8D206AC39C22}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16380" xr2:uid="{AD88AA4B-C132-0C4D-B7C9-8D206AC39C22}"/>
   </bookViews>
   <sheets>
     <sheet name="Leaf" sheetId="3" r:id="rId1"/>
@@ -20,7 +20,6 @@
     <externalReference r:id="rId3"/>
     <externalReference r:id="rId4"/>
     <externalReference r:id="rId5"/>
-    <externalReference r:id="rId6"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
@@ -364,7 +363,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -414,6 +413,9 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -437,6 +439,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="GFS-Linear"/>
@@ -451,88 +454,88 @@
       <sheetData sheetId="1"/>
       <sheetData sheetId="2">
         <row r="71">
-          <cell r="AJ71">
+          <cell r="AL71">
             <v>357.73817371239033</v>
           </cell>
         </row>
         <row r="72">
-          <cell r="AJ72">
+          <cell r="AL72">
             <v>451.98153105926428</v>
           </cell>
         </row>
         <row r="73">
-          <cell r="AJ73">
+          <cell r="AL73">
             <v>318.4117385185852</v>
           </cell>
         </row>
         <row r="74">
-          <cell r="AJ74">
+          <cell r="AL74">
             <v>230.6394891915813</v>
           </cell>
         </row>
         <row r="75">
-          <cell r="AJ75">
+          <cell r="AL75">
             <v>286.21365916523314</v>
           </cell>
         </row>
         <row r="76">
-          <cell r="AJ76">
+          <cell r="AL76">
             <v>202.30840866209519</v>
           </cell>
         </row>
         <row r="77">
-          <cell r="AJ77">
+          <cell r="AL77">
             <v>267.71075832927647</v>
           </cell>
         </row>
         <row r="78">
-          <cell r="AJ78">
+          <cell r="AL78">
             <v>88.571268184648915</v>
           </cell>
         </row>
         <row r="79">
-          <cell r="AJ79">
+          <cell r="AL79">
             <v>563.50735539320715</v>
           </cell>
         </row>
         <row r="80">
-          <cell r="AJ80">
+          <cell r="AL80">
             <v>843.6065588733702</v>
           </cell>
         </row>
         <row r="81">
-          <cell r="AJ81">
+          <cell r="AL81">
             <v>284.90499166962036</v>
           </cell>
         </row>
         <row r="82">
-          <cell r="AJ82">
+          <cell r="AL82">
             <v>304.80534510512013</v>
           </cell>
         </row>
         <row r="83">
-          <cell r="AJ83">
+          <cell r="AL83">
             <v>139.78364360646955</v>
           </cell>
         </row>
         <row r="84">
-          <cell r="AJ84">
+          <cell r="AL84">
             <v>390.72249733057782</v>
           </cell>
         </row>
         <row r="85">
-          <cell r="AJ85">
+          <cell r="AL85">
             <v>310.92474780645216</v>
           </cell>
         </row>
         <row r="86">
-          <cell r="AJ86">
+          <cell r="AL86">
             <v>311.78530890104531</v>
           </cell>
         </row>
-        <row r="88">
-          <cell r="AJ88">
-            <v>16.367130494667343</v>
+        <row r="87">
+          <cell r="AL87">
+            <v>45.143393429783053</v>
           </cell>
         </row>
       </sheetData>
@@ -549,6 +552,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Starch Data Template"/>
@@ -655,6 +659,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="GFS-Linear"/>
@@ -670,114 +675,90 @@
       <sheetData sheetId="2">
         <row r="71">
           <cell r="AJ71">
+            <v>4</v>
+          </cell>
+          <cell r="AK71">
             <v>465.21117651276387</v>
           </cell>
         </row>
         <row r="72">
-          <cell r="AJ72">
+          <cell r="AK72">
             <v>170.17176340344352</v>
           </cell>
         </row>
         <row r="73">
-          <cell r="AJ73">
+          <cell r="AK73">
             <v>340.29642713813917</v>
           </cell>
         </row>
         <row r="74">
-          <cell r="AJ74">
+          <cell r="AK74">
             <v>233.24838429981111</v>
           </cell>
         </row>
         <row r="75">
-          <cell r="AJ75">
+          <cell r="AK75">
             <v>237.98235002929687</v>
           </cell>
         </row>
         <row r="76">
-          <cell r="AJ76">
+          <cell r="AK76">
             <v>317.95879431137979</v>
           </cell>
         </row>
         <row r="77">
-          <cell r="AJ77">
+          <cell r="AK77">
             <v>493.70680903300189</v>
           </cell>
         </row>
         <row r="78">
-          <cell r="AJ78">
+          <cell r="AK78">
             <v>203.11059768711317</v>
           </cell>
         </row>
         <row r="79">
-          <cell r="AJ79">
+          <cell r="AK79">
             <v>884.0855677542321</v>
           </cell>
         </row>
         <row r="80">
-          <cell r="AJ80">
+          <cell r="AK80">
             <v>829.22196047482032</v>
           </cell>
         </row>
         <row r="81">
-          <cell r="AJ81">
+          <cell r="AK81">
             <v>231.22933122557191</v>
           </cell>
         </row>
         <row r="82">
-          <cell r="AJ82">
+          <cell r="AK82">
             <v>278.64077258566851</v>
           </cell>
         </row>
         <row r="83">
-          <cell r="AJ83">
+          <cell r="AK83">
             <v>284.39322165427473</v>
           </cell>
         </row>
         <row r="84">
-          <cell r="AJ84">
+          <cell r="AK84">
             <v>560.02660719257426</v>
           </cell>
         </row>
         <row r="85">
-          <cell r="AJ85">
+          <cell r="AK85">
             <v>697.33197880763078</v>
           </cell>
         </row>
         <row r="86">
-          <cell r="AJ86">
+          <cell r="AK86">
             <v>492.39845512222291</v>
           </cell>
         </row>
-      </sheetData>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink4.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="GFS-Linear"/>
-      <sheetName val="GFS in Assay Summary"/>
-      <sheetName val="GFS-Quad-Ending (2)"/>
-      <sheetName val="GFS-Quad-Ending"/>
-      <sheetName val="GFS-Quad"/>
-      <sheetName val="Sheet1"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2">
-        <row r="88">
-          <cell r="AJ88">
-            <v>60.963492730850888</v>
+        <row r="87">
+          <cell r="AK87">
+            <v>-27.031217596952501</v>
           </cell>
         </row>
       </sheetData>
@@ -1394,7 +1375,7 @@
         <v>112.20945996754307</v>
       </c>
       <c r="AA3" s="29">
-        <f t="shared" ref="AA3:AA17" si="8">Z3/Y3</f>
+        <f t="shared" ref="AA3:AA18" si="8">Z3/Y3</f>
         <v>0.21295552034224496</v>
       </c>
     </row>
@@ -2702,9 +2683,12 @@
       <c r="M18" s="4"/>
       <c r="N18" s="4"/>
       <c r="O18" s="4"/>
+      <c r="Y18" s="39"/>
+      <c r="Z18" s="40"/>
+      <c r="AA18" s="41"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="AA2:AA17">
+  <conditionalFormatting sqref="AA2:AA18">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -2720,7 +2704,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2231F396-29C4-F943-9364-FC14281A2FC0}">
-  <dimension ref="A1:AA18"/>
+  <dimension ref="A1:AA19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="5.6640625" bestFit="1" customWidth="1"/>
@@ -2851,7 +2835,7 @@
         <v>DOY 186: 07/05/22</v>
       </c>
       <c r="H2" s="6">
-        <f>'[1]GFS-Quad-Ending'!$AJ71</f>
+        <f>'[1]GFS-Quad-Ending'!$AL71</f>
         <v>357.73817371239033</v>
       </c>
       <c r="I2" s="7">
@@ -2859,7 +2843,7 @@
         <v>56.92460968948081</v>
       </c>
       <c r="J2" s="6">
-        <f>'[3]GFS-Quad-Ending (2)'!$AJ71</f>
+        <f>'[3]GFS-Quad-Ending (2)'!$AK71</f>
         <v>465.21117651276387</v>
       </c>
       <c r="K2" s="7">
@@ -2878,15 +2862,15 @@
         <v>32.299999999999997</v>
       </c>
       <c r="P2" s="11">
-        <f t="shared" ref="P2:P18" si="0">H2+I2</f>
+        <f>H2+I2</f>
         <v>414.66278340187114</v>
       </c>
       <c r="Q2" s="11">
-        <f t="shared" ref="Q2:Q18" si="1">J2+K2</f>
+        <f t="shared" ref="Q2:Q18" si="0">J2+K2</f>
         <v>1028.755536293052</v>
       </c>
       <c r="R2" s="11">
-        <f t="shared" ref="R2:R18" si="2">L2+M2</f>
+        <f t="shared" ref="R2:R18" si="1">L2+M2</f>
         <v>1155.8078842722391</v>
       </c>
       <c r="S2" s="11">
@@ -2942,11 +2926,11 @@
         <v>44747</v>
       </c>
       <c r="G3" s="37" t="str">
-        <f t="shared" ref="G3:G18" si="3">_xlfn.CONCAT("DOY ", C3, ": ", TEXT(F3,"mm/dd/yy"))</f>
+        <f t="shared" ref="G3:G18" si="2">_xlfn.CONCAT("DOY ", C3, ": ", TEXT(F3,"mm/dd/yy"))</f>
         <v>DOY 186: 07/05/22</v>
       </c>
       <c r="H3" s="6">
-        <f>'[1]GFS-Quad-Ending'!$AJ72</f>
+        <f>'[1]GFS-Quad-Ending'!$AL72</f>
         <v>451.98153105926428</v>
       </c>
       <c r="I3" s="7">
@@ -2954,7 +2938,7 @@
         <v>185.2936715334319</v>
       </c>
       <c r="J3" s="6">
-        <f>'[3]GFS-Quad-Ending (2)'!$AJ72</f>
+        <f>'[3]GFS-Quad-Ending (2)'!$AK72</f>
         <v>170.17176340344352</v>
       </c>
       <c r="K3" s="7">
@@ -2973,15 +2957,15 @@
         <v>77.2</v>
       </c>
       <c r="P3" s="11">
+        <f t="shared" ref="P2:P18" si="3">H3+I3</f>
+        <v>637.27520259269613</v>
+      </c>
+      <c r="Q3" s="11">
         <f t="shared" si="0"/>
-        <v>637.27520259269613</v>
-      </c>
-      <c r="Q3" s="11">
+        <v>395.56729235885507</v>
+      </c>
+      <c r="R3" s="11">
         <f t="shared" si="1"/>
-        <v>395.56729235885507</v>
-      </c>
-      <c r="R3" s="11">
-        <f t="shared" si="2"/>
         <v>393.18247748160707</v>
       </c>
       <c r="S3" s="11">
@@ -3037,11 +3021,11 @@
         <v>44747</v>
       </c>
       <c r="G4" s="37" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DOY 186: 07/05/22</v>
       </c>
       <c r="H4" s="6">
-        <f>'[1]GFS-Quad-Ending'!$AJ73</f>
+        <f>'[1]GFS-Quad-Ending'!$AL73</f>
         <v>318.4117385185852</v>
       </c>
       <c r="I4" s="7">
@@ -3049,7 +3033,7 @@
         <v>40.41494877630074</v>
       </c>
       <c r="J4" s="6">
-        <f>'[3]GFS-Quad-Ending (2)'!$AJ73</f>
+        <f>'[3]GFS-Quad-Ending (2)'!$AK73</f>
         <v>340.29642713813917</v>
       </c>
       <c r="K4" s="7">
@@ -3068,15 +3052,15 @@
         <v>177.5</v>
       </c>
       <c r="P4" s="11">
+        <f t="shared" si="3"/>
+        <v>358.82668729488591</v>
+      </c>
+      <c r="Q4" s="11">
         <f t="shared" si="0"/>
-        <v>358.82668729488591</v>
-      </c>
-      <c r="Q4" s="11">
+        <v>521.83523402347021</v>
+      </c>
+      <c r="R4" s="11">
         <f t="shared" si="1"/>
-        <v>521.83523402347021</v>
-      </c>
-      <c r="R4" s="11">
-        <f t="shared" si="2"/>
         <v>628.75303733562737</v>
       </c>
       <c r="S4" s="11">
@@ -3132,11 +3116,11 @@
         <v>44747</v>
       </c>
       <c r="G5" s="37" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DOY 186: 07/05/22</v>
       </c>
       <c r="H5" s="6">
-        <f>'[1]GFS-Quad-Ending'!$AJ74</f>
+        <f>'[1]GFS-Quad-Ending'!$AL74</f>
         <v>230.6394891915813</v>
       </c>
       <c r="I5" s="7">
@@ -3144,7 +3128,7 @@
         <v>213.27914004026843</v>
       </c>
       <c r="J5" s="6">
-        <f>'[3]GFS-Quad-Ending (2)'!$AJ74</f>
+        <f>'[3]GFS-Quad-Ending (2)'!$AK74</f>
         <v>233.24838429981111</v>
       </c>
       <c r="K5" s="7">
@@ -3163,15 +3147,15 @@
         <v>46.8</v>
       </c>
       <c r="P5" s="11">
+        <f t="shared" si="3"/>
+        <v>443.91862923184976</v>
+      </c>
+      <c r="Q5" s="11">
         <f t="shared" si="0"/>
-        <v>443.91862923184976</v>
-      </c>
-      <c r="Q5" s="11">
+        <v>363.31177972919954</v>
+      </c>
+      <c r="R5" s="11">
         <f t="shared" si="1"/>
-        <v>363.31177972919954</v>
-      </c>
-      <c r="R5" s="11">
-        <f t="shared" si="2"/>
         <v>889.59249770700649</v>
       </c>
       <c r="S5" s="11">
@@ -3227,11 +3211,11 @@
         <v>44747</v>
       </c>
       <c r="G6" s="37" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DOY 186: 07/05/22</v>
       </c>
       <c r="H6" s="6">
-        <f>'[1]GFS-Quad-Ending'!$AJ75</f>
+        <f>'[1]GFS-Quad-Ending'!$AL75</f>
         <v>286.21365916523314</v>
       </c>
       <c r="I6" s="7">
@@ -3239,7 +3223,7 @@
         <v>267.43122054523008</v>
       </c>
       <c r="J6" s="6">
-        <f>'[3]GFS-Quad-Ending (2)'!$AJ75</f>
+        <f>'[3]GFS-Quad-Ending (2)'!$AK75</f>
         <v>237.98235002929687</v>
       </c>
       <c r="K6" s="7">
@@ -3258,15 +3242,15 @@
         <v>419.7</v>
       </c>
       <c r="P6" s="11">
+        <f t="shared" si="3"/>
+        <v>553.64487971046321</v>
+      </c>
+      <c r="Q6" s="11">
         <f t="shared" si="0"/>
-        <v>553.64487971046321</v>
-      </c>
-      <c r="Q6" s="11">
+        <v>483.53985540571693</v>
+      </c>
+      <c r="R6" s="11">
         <f t="shared" si="1"/>
-        <v>483.53985540571693</v>
-      </c>
-      <c r="R6" s="11">
-        <f t="shared" si="2"/>
         <v>456.21635040169832</v>
       </c>
       <c r="S6" s="11">
@@ -3322,11 +3306,11 @@
         <v>44748</v>
       </c>
       <c r="G7" s="37" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DOY 187: 07/06/22</v>
       </c>
       <c r="H7" s="6">
-        <f>'[1]GFS-Quad-Ending'!$AJ76</f>
+        <f>'[1]GFS-Quad-Ending'!$AL76</f>
         <v>202.30840866209519</v>
       </c>
       <c r="I7" s="7">
@@ -3334,7 +3318,7 @@
         <v>131.24365010383582</v>
       </c>
       <c r="J7" s="6">
-        <f>'[3]GFS-Quad-Ending (2)'!$AJ76</f>
+        <f>'[3]GFS-Quad-Ending (2)'!$AK76</f>
         <v>317.95879431137979</v>
       </c>
       <c r="K7" s="7">
@@ -3353,15 +3337,15 @@
         <v>559.79999999999995</v>
       </c>
       <c r="P7" s="11">
+        <f t="shared" si="3"/>
+        <v>333.55205876593101</v>
+      </c>
+      <c r="Q7" s="11">
         <f t="shared" si="0"/>
-        <v>333.55205876593101</v>
-      </c>
-      <c r="Q7" s="11">
+        <v>499.0741191448783</v>
+      </c>
+      <c r="R7" s="11">
         <f t="shared" si="1"/>
-        <v>499.0741191448783</v>
-      </c>
-      <c r="R7" s="11">
-        <f t="shared" si="2"/>
         <v>847.6735187043073</v>
       </c>
       <c r="S7" s="11">
@@ -3417,11 +3401,11 @@
         <v>44748</v>
       </c>
       <c r="G8" s="37" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DOY 187: 07/06/22</v>
       </c>
       <c r="H8" s="6">
-        <f>'[1]GFS-Quad-Ending'!$AJ77</f>
+        <f>'[1]GFS-Quad-Ending'!$AL77</f>
         <v>267.71075832927647</v>
       </c>
       <c r="I8" s="7">
@@ -3429,7 +3413,7 @@
         <v>21.188792508147095</v>
       </c>
       <c r="J8" s="6">
-        <f>'[3]GFS-Quad-Ending (2)'!$AJ77</f>
+        <f>'[3]GFS-Quad-Ending (2)'!$AK77</f>
         <v>493.70680903300189</v>
       </c>
       <c r="K8" s="7">
@@ -3448,15 +3432,15 @@
         <v>9.8000000000000007</v>
       </c>
       <c r="P8" s="11">
+        <f t="shared" si="3"/>
+        <v>288.89955083742359</v>
+      </c>
+      <c r="Q8" s="11">
         <f t="shared" si="0"/>
-        <v>288.89955083742359</v>
-      </c>
-      <c r="Q8" s="11">
+        <v>628.8477983966286</v>
+      </c>
+      <c r="R8" s="11">
         <f t="shared" si="1"/>
-        <v>628.8477983966286</v>
-      </c>
-      <c r="R8" s="11">
-        <f t="shared" si="2"/>
         <v>440.037625188314</v>
       </c>
       <c r="S8" s="11">
@@ -3512,11 +3496,11 @@
         <v>44748</v>
       </c>
       <c r="G9" s="37" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DOY 187: 07/06/22</v>
       </c>
       <c r="H9" s="6">
-        <f>'[1]GFS-Quad-Ending'!$AJ78</f>
+        <f>'[1]GFS-Quad-Ending'!$AL78</f>
         <v>88.571268184648915</v>
       </c>
       <c r="I9" s="7">
@@ -3524,7 +3508,7 @@
         <v>10.263392850610167</v>
       </c>
       <c r="J9" s="6">
-        <f>'[3]GFS-Quad-Ending (2)'!$AJ78</f>
+        <f>'[3]GFS-Quad-Ending (2)'!$AK78</f>
         <v>203.11059768711317</v>
       </c>
       <c r="K9" s="7">
@@ -3543,15 +3527,15 @@
         <v>43.9</v>
       </c>
       <c r="P9" s="11">
+        <f t="shared" si="3"/>
+        <v>98.834661035259074</v>
+      </c>
+      <c r="Q9" s="11">
         <f t="shared" si="0"/>
-        <v>98.834661035259074</v>
-      </c>
-      <c r="Q9" s="11">
+        <v>288.78402846985568</v>
+      </c>
+      <c r="R9" s="11">
         <f t="shared" si="1"/>
-        <v>288.78402846985568</v>
-      </c>
-      <c r="R9" s="11">
-        <f t="shared" si="2"/>
         <v>135.62733566134267</v>
       </c>
       <c r="S9" s="11">
@@ -3607,11 +3591,11 @@
         <v>44770</v>
       </c>
       <c r="G10" s="37" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DOY 209: 07/28/22</v>
       </c>
       <c r="H10" s="6">
-        <f>'[1]GFS-Quad-Ending'!$AJ79</f>
+        <f>'[1]GFS-Quad-Ending'!$AL79</f>
         <v>563.50735539320715</v>
       </c>
       <c r="I10" s="7">
@@ -3619,7 +3603,7 @@
         <v>28.643477715767389</v>
       </c>
       <c r="J10" s="6">
-        <f>'[3]GFS-Quad-Ending (2)'!$AJ79</f>
+        <f>'[3]GFS-Quad-Ending (2)'!$AK79</f>
         <v>884.0855677542321</v>
       </c>
       <c r="K10" s="7">
@@ -3638,15 +3622,15 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="P10" s="11">
+        <f t="shared" si="3"/>
+        <v>592.15083310897455</v>
+      </c>
+      <c r="Q10" s="11">
         <f t="shared" si="0"/>
-        <v>592.15083310897455</v>
-      </c>
-      <c r="Q10" s="11">
+        <v>981.6620113954358</v>
+      </c>
+      <c r="R10" s="11">
         <f t="shared" si="1"/>
-        <v>981.6620113954358</v>
-      </c>
-      <c r="R10" s="11">
-        <f t="shared" si="2"/>
         <v>1371.3569954477159</v>
       </c>
       <c r="S10" s="11">
@@ -3702,11 +3686,11 @@
         <v>44770</v>
       </c>
       <c r="G11" s="37" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DOY 209: 07/28/22</v>
       </c>
       <c r="H11" s="6">
-        <f>'[1]GFS-Quad-Ending'!$AJ80</f>
+        <f>'[1]GFS-Quad-Ending'!$AL80</f>
         <v>843.6065588733702</v>
       </c>
       <c r="I11" s="7">
@@ -3714,7 +3698,7 @@
         <v>116.81975866661671</v>
       </c>
       <c r="J11" s="6">
-        <f>'[3]GFS-Quad-Ending (2)'!$AJ80</f>
+        <f>'[3]GFS-Quad-Ending (2)'!$AK80</f>
         <v>829.22196047482032</v>
       </c>
       <c r="K11" s="7">
@@ -3733,15 +3717,15 @@
         <v>59.3</v>
       </c>
       <c r="P11" s="11">
+        <f t="shared" si="3"/>
+        <v>960.42631753998694</v>
+      </c>
+      <c r="Q11" s="11">
         <f t="shared" si="0"/>
-        <v>960.42631753998694</v>
-      </c>
-      <c r="Q11" s="11">
+        <v>876.87231564837771</v>
+      </c>
+      <c r="R11" s="11">
         <f t="shared" si="1"/>
-        <v>876.87231564837771</v>
-      </c>
-      <c r="R11" s="11">
-        <f t="shared" si="2"/>
         <v>643.08552167125174</v>
       </c>
       <c r="S11" s="11">
@@ -3797,11 +3781,11 @@
         <v>44797</v>
       </c>
       <c r="G12" s="37" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DOY 236: 08/24/22</v>
       </c>
       <c r="H12" s="6">
-        <f>'[1]GFS-Quad-Ending'!$AJ81</f>
+        <f>'[1]GFS-Quad-Ending'!$AL81</f>
         <v>284.90499166962036</v>
       </c>
       <c r="I12" s="7">
@@ -3809,7 +3793,7 @@
         <v>104.29614874178957</v>
       </c>
       <c r="J12" s="6">
-        <f>'[3]GFS-Quad-Ending (2)'!$AJ81</f>
+        <f>'[3]GFS-Quad-Ending (2)'!$AK81</f>
         <v>231.22933122557191</v>
       </c>
       <c r="K12" s="7">
@@ -3828,15 +3812,15 @@
         <v>132.5</v>
       </c>
       <c r="P12" s="11">
+        <f t="shared" si="3"/>
+        <v>389.20114041140994</v>
+      </c>
+      <c r="Q12" s="11">
         <f t="shared" si="0"/>
-        <v>389.20114041140994</v>
-      </c>
-      <c r="Q12" s="11">
+        <v>315.23914410201832</v>
+      </c>
+      <c r="R12" s="11">
         <f t="shared" si="1"/>
-        <v>315.23914410201832</v>
-      </c>
-      <c r="R12" s="11">
-        <f t="shared" si="2"/>
         <v>546.85201669573576</v>
       </c>
       <c r="S12" s="11">
@@ -3892,11 +3876,11 @@
         <v>44797</v>
       </c>
       <c r="G13" s="37" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DOY 236: 08/24/22</v>
       </c>
       <c r="H13" s="6">
-        <f>'[1]GFS-Quad-Ending'!$AJ82</f>
+        <f>'[1]GFS-Quad-Ending'!$AL82</f>
         <v>304.80534510512013</v>
       </c>
       <c r="I13" s="7">
@@ -3904,7 +3888,7 @@
         <v>62.549959164553528</v>
       </c>
       <c r="J13" s="6">
-        <f>'[3]GFS-Quad-Ending (2)'!$AJ82</f>
+        <f>'[3]GFS-Quad-Ending (2)'!$AK82</f>
         <v>278.64077258566851</v>
       </c>
       <c r="K13" s="7">
@@ -3923,15 +3907,15 @@
         <v>186.3</v>
       </c>
       <c r="P13" s="11">
+        <f t="shared" si="3"/>
+        <v>367.35530426967364</v>
+      </c>
+      <c r="Q13" s="11">
         <f t="shared" si="0"/>
-        <v>367.35530426967364</v>
-      </c>
-      <c r="Q13" s="11">
+        <v>391.86012590301812</v>
+      </c>
+      <c r="R13" s="11">
         <f t="shared" si="1"/>
-        <v>391.86012590301812</v>
-      </c>
-      <c r="R13" s="11">
-        <f t="shared" si="2"/>
         <v>517.44348296366252</v>
       </c>
       <c r="S13" s="11">
@@ -3987,11 +3971,11 @@
         <v>44797</v>
       </c>
       <c r="G14" s="37" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DOY 236: 08/24/22</v>
       </c>
       <c r="H14" s="6">
-        <f>'[1]GFS-Quad-Ending'!$AJ83</f>
+        <f>'[1]GFS-Quad-Ending'!$AL83</f>
         <v>139.78364360646955</v>
       </c>
       <c r="I14" s="7">
@@ -3999,7 +3983,7 @@
         <v>334.1909380485165</v>
       </c>
       <c r="J14" s="6">
-        <f>'[3]GFS-Quad-Ending (2)'!$AJ83</f>
+        <f>'[3]GFS-Quad-Ending (2)'!$AK83</f>
         <v>284.39322165427473</v>
       </c>
       <c r="K14" s="7">
@@ -4018,15 +4002,15 @@
         <v>113.8</v>
       </c>
       <c r="P14" s="11">
+        <f t="shared" si="3"/>
+        <v>473.97458165498608</v>
+      </c>
+      <c r="Q14" s="11">
         <f t="shared" si="0"/>
-        <v>473.97458165498608</v>
-      </c>
-      <c r="Q14" s="11">
+        <v>412.58094092118904</v>
+      </c>
+      <c r="R14" s="11">
         <f t="shared" si="1"/>
-        <v>412.58094092118904</v>
-      </c>
-      <c r="R14" s="11">
-        <f t="shared" si="2"/>
         <v>521.46298908168706</v>
       </c>
       <c r="S14" s="11">
@@ -4082,11 +4066,11 @@
         <v>44819</v>
       </c>
       <c r="G15" s="37" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DOY 258: 09/15/22</v>
       </c>
       <c r="H15" s="6">
-        <f>'[1]GFS-Quad-Ending'!$AJ84</f>
+        <f>'[1]GFS-Quad-Ending'!$AL84</f>
         <v>390.72249733057782</v>
       </c>
       <c r="I15" s="7">
@@ -4094,7 +4078,7 @@
         <v>-1.5308150136254652</v>
       </c>
       <c r="J15" s="6">
-        <f>'[3]GFS-Quad-Ending (2)'!$AJ84</f>
+        <f>'[3]GFS-Quad-Ending (2)'!$AK84</f>
         <v>560.02660719257426</v>
       </c>
       <c r="K15" s="7">
@@ -4113,15 +4097,15 @@
         <v>38.6</v>
       </c>
       <c r="P15" s="11">
+        <f t="shared" si="3"/>
+        <v>389.19168231695238</v>
+      </c>
+      <c r="Q15" s="11">
         <f t="shared" si="0"/>
-        <v>389.19168231695238</v>
-      </c>
-      <c r="Q15" s="11">
+        <v>591.85151503934776</v>
+      </c>
+      <c r="R15" s="11">
         <f t="shared" si="1"/>
-        <v>591.85151503934776</v>
-      </c>
-      <c r="R15" s="11">
-        <f t="shared" si="2"/>
         <v>508.33027243293543</v>
       </c>
       <c r="S15" s="11">
@@ -4177,11 +4161,11 @@
         <v>44819</v>
       </c>
       <c r="G16" s="37" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DOY 258: 09/15/22</v>
       </c>
       <c r="H16" s="6">
-        <f>'[1]GFS-Quad-Ending'!$AJ85</f>
+        <f>'[1]GFS-Quad-Ending'!$AL85</f>
         <v>310.92474780645216</v>
       </c>
       <c r="I16" s="7">
@@ -4189,7 +4173,7 @@
         <v>-5.6291934515707824</v>
       </c>
       <c r="J16" s="6">
-        <f>'[3]GFS-Quad-Ending (2)'!$AJ85</f>
+        <f>'[3]GFS-Quad-Ending (2)'!$AK85</f>
         <v>697.33197880763078</v>
       </c>
       <c r="K16" s="7">
@@ -4208,15 +4192,15 @@
         <v>290.10000000000002</v>
       </c>
       <c r="P16" s="11">
+        <f t="shared" si="3"/>
+        <v>305.2955543548814</v>
+      </c>
+      <c r="Q16" s="11">
         <f t="shared" si="0"/>
-        <v>305.2955543548814</v>
-      </c>
-      <c r="Q16" s="11">
+        <v>702.71528662606681</v>
+      </c>
+      <c r="R16" s="11">
         <f t="shared" si="1"/>
-        <v>702.71528662606681</v>
-      </c>
-      <c r="R16" s="11">
-        <f t="shared" si="2"/>
         <v>328.98862685756023</v>
       </c>
       <c r="S16" s="11">
@@ -4272,11 +4256,11 @@
         <v>44819</v>
       </c>
       <c r="G17" s="37" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DOY 258: 09/15/22</v>
       </c>
       <c r="H17" s="6">
-        <f>'[1]GFS-Quad-Ending'!$AJ86</f>
+        <f>'[1]GFS-Quad-Ending'!$AL86</f>
         <v>311.78530890104531</v>
       </c>
       <c r="I17" s="7">
@@ -4284,7 +4268,7 @@
         <v>-1.1089238686873388</v>
       </c>
       <c r="J17" s="6">
-        <f>'[3]GFS-Quad-Ending (2)'!$AJ86</f>
+        <f>'[3]GFS-Quad-Ending (2)'!$AK86</f>
         <v>492.39845512222291</v>
       </c>
       <c r="K17" s="7">
@@ -4303,15 +4287,15 @@
         <v>74.8</v>
       </c>
       <c r="P17" s="11">
+        <f t="shared" si="3"/>
+        <v>310.67638503235798</v>
+      </c>
+      <c r="Q17" s="11">
         <f t="shared" si="0"/>
-        <v>310.67638503235798</v>
-      </c>
-      <c r="Q17" s="11">
+        <v>516.20731643414774</v>
+      </c>
+      <c r="R17" s="11">
         <f t="shared" si="1"/>
-        <v>516.20731643414774</v>
-      </c>
-      <c r="R17" s="11">
-        <f t="shared" si="2"/>
         <v>693.07788229297842</v>
       </c>
       <c r="S17" s="11">
@@ -4367,20 +4351,20 @@
         <v>44839</v>
       </c>
       <c r="G18" s="37" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DOY 278: 10/05/22</v>
       </c>
-      <c r="H18" s="8">
-        <f>'[1]GFS-Quad-Ending'!$AJ88</f>
-        <v>16.367130494667343</v>
+      <c r="H18" s="6">
+        <f>'[1]GFS-Quad-Ending'!$AL87</f>
+        <v>45.143393429783053</v>
       </c>
       <c r="I18" s="9">
         <f>'[2]Starch Data Template'!$P71</f>
         <v>-4.8437083701565822</v>
       </c>
-      <c r="J18" s="8">
-        <f>'[4]GFS-Quad-Ending (2)'!$AJ$88</f>
-        <v>60.963492730850888</v>
+      <c r="J18" s="6">
+        <f>'[3]GFS-Quad-Ending (2)'!$AK87</f>
+        <v>-27.031217596952501</v>
       </c>
       <c r="K18" s="9">
         <v>36.897564145831879</v>
@@ -4398,15 +4382,15 @@
         <v>0</v>
       </c>
       <c r="P18" s="11">
+        <f t="shared" si="3"/>
+        <v>40.299685059626469</v>
+      </c>
+      <c r="Q18" s="11">
         <f t="shared" si="0"/>
-        <v>11.523422124510761</v>
-      </c>
-      <c r="Q18" s="11">
+        <v>9.8663465488793776</v>
+      </c>
+      <c r="R18" s="11">
         <f t="shared" si="1"/>
-        <v>97.861056876682767</v>
-      </c>
-      <c r="R18" s="11">
-        <f t="shared" si="2"/>
         <v>213.96375340002535</v>
       </c>
       <c r="S18" s="11">
@@ -4441,6 +4425,10 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
+    </row>
+    <row r="19" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="Y19" s="39"/>
+      <c r="Z19" s="40"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>